<commit_message>
Update dashboard with correlation stat and final formatting
</commit_message>
<xml_diff>
--- a/nba team financials.xlsx
+++ b/nba team financials.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/twandon/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D465D3B1-B685-1849-AFF3-2CBE8D2FBC46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C3DF6C77-F98B-5942-97E6-E86F4F05C915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{060D5569-2AC9-B04F-841D-CEA7829076CD}"/>
   </bookViews>
   <sheets>
-    <sheet name="nba_team_financials" sheetId="1" r:id="rId1"/>
+    <sheet name="Data" sheetId="1" r:id="rId1"/>
     <sheet name="Calculations" sheetId="2" r:id="rId2"/>
     <sheet name="Rankings" sheetId="3" r:id="rId3"/>
     <sheet name="Dashboard" sheetId="6" r:id="rId4"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="96">
   <si>
     <t>2025-26 NBA Season</t>
   </si>
@@ -327,6 +327,9 @@
   </si>
   <si>
     <t>#2 spend ($232.0M), league-worst 17 wins</t>
+  </si>
+  <si>
+    <t>Key Question: Does spending more money on players actually make an NBA team win more?</t>
   </si>
 </sst>
 </file>
@@ -343,7 +346,7 @@
     <numFmt numFmtId="168" formatCode="0.0%"/>
     <numFmt numFmtId="169" formatCode="&quot;$&quot;0.0&quot;M&quot;"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -434,6 +437,20 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
       <sz val="16"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -691,7 +708,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -792,15 +809,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="10" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="10" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="10" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="169" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -872,6 +880,21 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="10" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1383,7 +1406,7 @@
                         <a:cs typeface="+mn-cs"/>
                       </a:defRPr>
                     </a:pPr>
-                    <a:fld id="{D88DDE85-15C9-0E4F-9367-9D9861A67434}" type="CELLRANGE">
+                    <a:fld id="{0B6D3822-4166-4941-9F10-34006DEAADC7}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr>
                         <a:defRPr/>
@@ -1449,7 +1472,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{37E722F0-2037-0042-83B7-AD285697A81C}" type="CELLRANGE">
+                    <a:fld id="{54AB3A83-D2B2-3249-B332-44BDD9710AF8}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1489,7 +1512,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{F9C6B634-9FC7-654E-A599-BEF255F27446}" type="CELLRANGE">
+                    <a:fld id="{A8E6CECD-2133-2A43-BEBD-52C446C4399C}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1528,7 +1551,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{D2DBB18D-FEF5-794C-9AF1-84F4CA270E83}" type="CELLRANGE">
+                    <a:fld id="{99B681EB-D59D-0943-93BA-9408FEE7355B}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1561,7 +1584,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{6EC94484-431C-B64B-A1EF-67225ECB497F}" type="CELLRANGE">
+                    <a:fld id="{F2EA1EE5-581B-BE47-AEDA-CCF39245E42E}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1635,7 +1658,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>(nba_team_financials!$A$11,nba_team_financials!$A$12,nba_team_financials!$A$23,nba_team_financials!$A$29,nba_team_financials!$A$32)</c:f>
+              <c:f>(Data!$A$11,Data!$A$12,Data!$A$23,Data!$A$29,Data!$A$32)</c:f>
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
@@ -1658,7 +1681,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>(nba_team_financials!$E$11,nba_team_financials!$E$12,nba_team_financials!$E$23,nba_team_financials!$E$29,nba_team_financials!$E$32)</c:f>
+              <c:f>(Data!$E$11,Data!$E$12,Data!$E$23,Data!$E$29,Data!$E$32)</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -1683,7 +1706,7 @@
           <c:extLst>
             <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
               <c15:datalabelsRange>
-                <c15:f>(nba_team_financials!$B$11,nba_team_financials!$B$12,nba_team_financials!$B$23,nba_team_financials!$B$29,nba_team_financials!$B$32)</c15:f>
+                <c15:f>(Data!$B$11,Data!$B$12,Data!$B$23,Data!$B$29,Data!$B$32)</c15:f>
                 <c15:dlblRangeCache>
                   <c:ptCount val="5"/>
                   <c:pt idx="0">
@@ -3043,13 +3066,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>744003</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:row>17</xdr:row>
       <xdr:rowOff>28727</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>787401</xdr:colOff>
-      <xdr:row>29</xdr:row>
+      <xdr:row>31</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -3081,13 +3104,13 @@
     <xdr:from>
       <xdr:col>8</xdr:col>
       <xdr:colOff>190947</xdr:colOff>
-      <xdr:row>14</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>149841</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>736601</xdr:colOff>
-      <xdr:row>29</xdr:row>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>31</xdr:row>
       <xdr:rowOff>139701</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -3117,9 +3140,9 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>16</xdr:col>
+      <xdr:col>14</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>32</xdr:row>
+      <xdr:row>34</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="184731" cy="264431"/>
@@ -3174,7 +3197,7 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>31</xdr:row>
+      <xdr:row>33</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="9225280" cy="1351279"/>
@@ -3229,13 +3252,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>762001</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:row>32</xdr:row>
       <xdr:rowOff>118534</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>558801</xdr:colOff>
-      <xdr:row>40</xdr:row>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>42</xdr:row>
       <xdr:rowOff>84667</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -3286,150 +3309,191 @@
         <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
         <a:lstStyle/>
         <a:p>
-          <a:pPr algn="l">
+          <a:pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
             <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
           </a:pPr>
           <a:r>
-            <a:rPr lang="en-US" b="1" i="0">
+            <a:rPr lang="en-US" sz="1050" b="1" i="0">
               <a:solidFill>
-                <a:srgbClr val="000000"/>
+                <a:schemeClr val="dk1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
               <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
             </a:rPr>
             <a:t>Insights &amp; Key Findings</a:t>
           </a:r>
         </a:p>
         <a:p>
-          <a:pPr algn="l">
-            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:buChar char="•"/>
-          </a:pPr>
           <a:r>
-            <a:rPr lang="en-US" b="1" i="0">
+            <a:rPr lang="en-US" sz="1050" b="1" i="0">
               <a:solidFill>
-                <a:srgbClr val="000000"/>
+                <a:schemeClr val="dk1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
               <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>The Golden State Paradox (Business vs. On-Court Efficiency):</a:t>
+            <a:t>1. </a:t>
           </a:r>
-          <a:endParaRPr lang="en-US" b="0" i="0">
+          <a:r>
+            <a:rPr lang="en-US" sz="1050" b="1" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>Golden State: Strong Business Performance, Weak On-Court Conversion</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1050" b="0" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>Golden State ranked #1 in Revenue-to-Payroll, generating $3.76 in revenue for every $1 of payroll. The Warriors generated $880M in revenue while carrying the NBA's highest payroll at $234.2M. Despite that financial strength, they finished 37–45 with a 45.1% win percentage. The result shows that strong revenue generation does not necessarily translate into competitive success.</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1050" b="0" i="0">
             <a:solidFill>
-              <a:srgbClr val="000000"/>
+              <a:schemeClr val="dk1"/>
             </a:solidFill>
             <a:effectLst/>
             <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            <a:ea typeface="+mn-ea"/>
             <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:pPr algn="l">
-            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:buChar char="•"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" b="0" i="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Golden State ranked #1 in financial efficiency due to league-leading revenue generation ($880M), but posted only a 45.1% win percentage on a $234.2M payroll (#1 spending in the NBA). Excellent revenue leverage did not translate to winning games, directly justifying why the scoring model weights competitive performance (25%) alongside financial metrics.</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l">
-            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:buChar char="•"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" b="1" i="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Spending Does Not Guarantee Results (Capital Misallocation):</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" b="0" i="0">
+          <a:endParaRPr lang="en-US" sz="1050" b="0" i="0">
             <a:solidFill>
-              <a:srgbClr val="000000"/>
+              <a:schemeClr val="dk1"/>
             </a:solidFill>
             <a:effectLst/>
             <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            <a:ea typeface="+mn-ea"/>
             <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:pPr algn="l">
-            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:buChar char="•"/>
-          </a:pPr>
           <a:r>
-            <a:rPr lang="en-US" b="0" i="0">
+            <a:rPr lang="en-US" sz="1050" b="1" i="0">
               <a:solidFill>
-                <a:srgbClr val="000000"/>
+                <a:schemeClr val="dk1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
               <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>The Washington Wizards committed $232.0M in payroll (#2 in NBA spending) but finished dead last (#30 Overall) with a league-worst 17 wins. Conversely, the San Antonio Spurs maintained a low payroll ($184.0M, #25 in spending) while securing #4 Overall Efficiency and 62 wins (#2 Win %), proving disciplined roster construction creates superior value over raw capital deployment.</a:t>
+            <a:t>2. </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1050" b="1" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>Spending Does Not Guarantee Wins</a:t>
           </a:r>
         </a:p>
         <a:p>
-          <a:pPr algn="l">
-            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:buChar char="•"/>
-          </a:pPr>
           <a:r>
-            <a:rPr lang="en-US" b="1" i="0">
+            <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
               <a:solidFill>
-                <a:srgbClr val="000000"/>
+                <a:schemeClr val="dk1"/>
               </a:solidFill>
               <a:effectLst/>
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Oklahoma City Thunder: The Model Franchise:</a:t>
+            <a:t>Washington ranked #2 in payroll at $232.0M but finished 30th overall with a 17–65 record. In contrast, San Antonio spent $184.0M, ranked 25th in payroll, and finished 4th overall with 62 wins. The comparison highlights the gap between total spending and spending efficiency. Across all 30 teams, payroll showed only a weak statistical relationship with wins (correlation ≈ 0.17), confirming this pattern holds league-wide, not just in isolated cases.</a:t>
           </a:r>
-          <a:endParaRPr lang="en-US" b="0" i="0">
+          <a:endParaRPr lang="en-US" sz="1050" b="0" i="0">
             <a:solidFill>
-              <a:srgbClr val="000000"/>
+              <a:schemeClr val="dk1"/>
             </a:solidFill>
             <a:effectLst/>
             <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            <a:ea typeface="+mn-ea"/>
             <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:pPr algn="l">
-            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:buChar char="•"/>
-          </a:pPr>
           <a:r>
-            <a:rPr lang="en-US" b="0" i="0">
+            <a:rPr lang="en-US" sz="1050" b="1" i="0">
               <a:solidFill>
-                <a:srgbClr val="000000"/>
+                <a:schemeClr val="dk1"/>
               </a:solidFill>
               <a:effectLst/>
               <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
               <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>OKC posted the league's top winning percentage (78.0% / 64–18 record) while simultaneously ranking #1 in Wins per $1M Payroll (0.340). They represent the purest example in the dataset of financial discipline translating directly into elite competitive output.</a:t>
+            <a:t>3. </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1050" b="1" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>Oklahoma City: Strongest Example of Efficient Winning</a:t>
           </a:r>
         </a:p>
         <a:p>
-          <a:endParaRPr lang="en-US" sz="1100">
+          <a:r>
+            <a:rPr lang="en-US" sz="1050" b="0" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>Oklahoma City ranked #1 in Win % at 78.0% and #1 in Wins per $1M Payroll at 0.340. The Thunder won 64 games while maintaining a relatively modest $188.1M payroll. Their results represent the strongest combination of competitive performance and payroll efficiency in the dataset.</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1050" b="0" i="0">
+            <a:solidFill>
+              <a:schemeClr val="dk1"/>
+            </a:solidFill>
+            <a:effectLst/>
             <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            <a:ea typeface="+mn-ea"/>
             <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
           </a:endParaRPr>
         </a:p>
@@ -3786,7 +3850,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
@@ -3797,34 +3861,34 @@
       <c r="G1" s="3"/>
       <c r="H1" s="3"/>
       <c r="I1" s="19"/>
-      <c r="J1" s="47" t="s">
+      <c r="J1" s="44" t="s">
         <v>65</v>
       </c>
       <c r="K1" s="3"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A2" s="47" t="s">
+      <c r="A2" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="48" t="s">
+      <c r="B2" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="47" t="s">
+      <c r="C2" s="44" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="47" t="s">
+      <c r="D2" s="44" t="s">
         <v>42</v>
       </c>
-      <c r="E2" s="49" t="s">
+      <c r="E2" s="46" t="s">
         <v>78</v>
       </c>
-      <c r="F2" s="47" t="s">
+      <c r="F2" s="44" t="s">
         <v>43</v>
       </c>
-      <c r="G2" s="47" t="s">
+      <c r="G2" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="47" t="s">
+      <c r="H2" s="44" t="s">
         <v>5</v>
       </c>
       <c r="I2" s="1"/>
@@ -4669,54 +4733,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="47" t="s">
+      <c r="B1" s="44" t="s">
         <v>44</v>
       </c>
-      <c r="C1" s="47" t="s">
+      <c r="C1" s="44" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="47" t="s">
+      <c r="D1" s="44" t="s">
         <v>45</v>
       </c>
-      <c r="E1" s="47" t="s">
+      <c r="E1" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="50"/>
-      <c r="G1" s="47" t="s">
+      <c r="F1" s="47"/>
+      <c r="G1" s="44" t="s">
         <v>47</v>
       </c>
-      <c r="H1" s="47" t="s">
+      <c r="H1" s="44" t="s">
         <v>48</v>
       </c>
-      <c r="I1" s="47" t="s">
+      <c r="I1" s="44" t="s">
         <v>54</v>
       </c>
-      <c r="J1" s="47" t="s">
+      <c r="J1" s="44" t="s">
         <v>61</v>
       </c>
-      <c r="K1" s="50"/>
+      <c r="K1" s="47"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="5">
-        <f>nba_team_financials!C3/nba_team_financials!E3</f>
+        <f>Data!C3/Data!E3</f>
         <v>10369565.217391305</v>
       </c>
       <c r="C2" s="6">
-        <f>nba_team_financials!E3/(nba_team_financials!B3/1000000)</f>
+        <f>Data!E3/(Data!B3/1000000)</f>
         <v>0.23802675858528755</v>
       </c>
       <c r="D2" s="4">
-        <f>nba_team_financials!C3/nba_team_financials!B3</f>
+        <f>Data!C3/Data!B3</f>
         <v>2.4682339966343947</v>
       </c>
       <c r="E2" s="24">
-        <f>nba_team_financials!G3</f>
+        <f>Data!G3</f>
         <v>0.56100000000000005</v>
       </c>
       <c r="G2" s="3" t="s">
@@ -4738,19 +4802,19 @@
         <v>7</v>
       </c>
       <c r="B3" s="5">
-        <f>nba_team_financials!C4/nba_team_financials!E4</f>
+        <f>Data!C4/Data!E4</f>
         <v>8178571.4285714282</v>
       </c>
       <c r="C3" s="6">
-        <f>nba_team_financials!E4/(nba_team_financials!B4/1000000)</f>
+        <f>Data!E4/(Data!B4/1000000)</f>
         <v>0.28787881716516106</v>
       </c>
       <c r="D3" s="4">
-        <f>nba_team_financials!C4/nba_team_financials!B4</f>
+        <f>Data!C4/Data!B4</f>
         <v>2.3544374689579244</v>
       </c>
       <c r="E3" s="24">
-        <f>nba_team_financials!G4</f>
+        <f>Data!G4</f>
         <v>0.68300000000000005</v>
       </c>
       <c r="G3" s="3" t="s">
@@ -4772,19 +4836,19 @@
         <v>8</v>
       </c>
       <c r="B4" s="5">
-        <f>nba_team_financials!C5/nba_team_financials!E5</f>
+        <f>Data!C5/Data!E5</f>
         <v>20100000</v>
       </c>
       <c r="C4" s="6">
-        <f>nba_team_financials!E5/(nba_team_financials!B5/1000000)</f>
+        <f>Data!E5/(Data!B5/1000000)</f>
         <v>0.13248511768176058</v>
       </c>
       <c r="D4" s="4">
-        <f>nba_team_financials!C5/nba_team_financials!B5</f>
+        <f>Data!C5/Data!B5</f>
         <v>2.6629508654033875</v>
       </c>
       <c r="E4" s="24">
-        <f>nba_team_financials!G5</f>
+        <f>Data!G5</f>
         <v>0.24399999999999999</v>
       </c>
       <c r="G4" s="3" t="s">
@@ -4806,19 +4870,19 @@
         <v>9</v>
       </c>
       <c r="B5" s="5">
-        <f>nba_team_financials!C6/nba_team_financials!E6</f>
+        <f>Data!C6/Data!E6</f>
         <v>7454545.4545454541</v>
       </c>
       <c r="C5" s="6">
-        <f>nba_team_financials!E6/(nba_team_financials!B6/1000000)</f>
+        <f>Data!E6/(Data!B6/1000000)</f>
         <v>0.23938236130003732</v>
       </c>
       <c r="D5" s="4">
-        <f>nba_team_financials!C6/nba_team_financials!B6</f>
+        <f>Data!C6/Data!B6</f>
         <v>1.7844866933275507</v>
       </c>
       <c r="E5" s="24">
-        <f>nba_team_financials!G6</f>
+        <f>Data!G6</f>
         <v>0.53700000000000003</v>
       </c>
       <c r="G5" s="3" t="s">
@@ -4840,19 +4904,19 @@
         <v>10</v>
       </c>
       <c r="B6" s="5">
-        <f>nba_team_financials!C7/nba_team_financials!E7</f>
+        <f>Data!C7/Data!E7</f>
         <v>14000000</v>
       </c>
       <c r="C6" s="6">
-        <f>nba_team_financials!E7/(nba_team_financials!B7/1000000)</f>
+        <f>Data!E7/(Data!B7/1000000)</f>
         <v>0.16518068787749748</v>
       </c>
       <c r="D6" s="4">
-        <f>nba_team_financials!C7/nba_team_financials!B7</f>
+        <f>Data!C7/Data!B7</f>
         <v>2.3125296302849647</v>
       </c>
       <c r="E6" s="24">
-        <f>nba_team_financials!G7</f>
+        <f>Data!G7</f>
         <v>0.378</v>
       </c>
       <c r="G6" s="3" t="s">
@@ -4873,19 +4937,19 @@
         <v>11</v>
       </c>
       <c r="B7" s="5">
-        <f>nba_team_financials!C8/nba_team_financials!E8</f>
+        <f>Data!C8/Data!E8</f>
         <v>8461538.461538462</v>
       </c>
       <c r="C7" s="6">
-        <f>nba_team_financials!E8/(nba_team_financials!B8/1000000)</f>
+        <f>Data!E8/(Data!B8/1000000)</f>
         <v>0.22990338266131469</v>
       </c>
       <c r="D7" s="4">
-        <f>nba_team_financials!C8/nba_team_financials!B8</f>
+        <f>Data!C8/Data!B8</f>
         <v>1.945336314826509</v>
       </c>
       <c r="E7" s="24">
-        <f>nba_team_financials!G8</f>
+        <f>Data!G8</f>
         <v>0.63400000000000001</v>
       </c>
       <c r="G7" s="3" t="s">
@@ -4906,19 +4970,19 @@
         <v>12</v>
       </c>
       <c r="B8" s="5">
-        <f>nba_team_financials!C9/nba_team_financials!E9</f>
+        <f>Data!C9/Data!E9</f>
         <v>15653846.153846154</v>
       </c>
       <c r="C8" s="6">
-        <f>nba_team_financials!E9/(nba_team_financials!B9/1000000)</f>
+        <f>Data!E9/(Data!B9/1000000)</f>
         <v>0.12975837045046565</v>
       </c>
       <c r="D8" s="4">
-        <f>nba_team_financials!C9/nba_team_financials!B9</f>
+        <f>Data!C9/Data!B9</f>
         <v>2.0312175682053666</v>
       </c>
       <c r="E8" s="24">
-        <f>nba_team_financials!G9</f>
+        <f>Data!G9</f>
         <v>0.317</v>
       </c>
     </row>
@@ -4927,19 +4991,19 @@
         <v>13</v>
       </c>
       <c r="B9" s="5">
-        <f>nba_team_financials!C10/nba_team_financials!E10</f>
+        <f>Data!C10/Data!E10</f>
         <v>6740740.7407407407</v>
       </c>
       <c r="C9" s="6">
-        <f>nba_team_financials!E10/(nba_team_financials!B10/1000000)</f>
+        <f>Data!E10/(Data!B10/1000000)</f>
         <v>0.26899946322153406</v>
       </c>
       <c r="D9" s="4">
-        <f>nba_team_financials!C10/nba_team_financials!B10</f>
+        <f>Data!C10/Data!B10</f>
         <v>1.8132556409747853</v>
       </c>
       <c r="E9" s="24">
-        <f>nba_team_financials!G10</f>
+        <f>Data!G10</f>
         <v>0.65900000000000003</v>
       </c>
     </row>
@@ -4948,19 +5012,19 @@
         <v>14</v>
       </c>
       <c r="B10" s="5">
-        <f>nba_team_financials!C11/nba_team_financials!E11</f>
+        <f>Data!C11/Data!E11</f>
         <v>5350000</v>
       </c>
       <c r="C10" s="6">
-        <f>nba_team_financials!E11/(nba_team_financials!B11/1000000)</f>
+        <f>Data!E11/(Data!B11/1000000)</f>
         <v>0.31074798505697881</v>
       </c>
       <c r="D10" s="4">
-        <f>nba_team_financials!C11/nba_team_financials!B11</f>
+        <f>Data!C11/Data!B11</f>
         <v>1.6625017200548364</v>
       </c>
       <c r="E10" s="24">
-        <f>nba_team_financials!G11</f>
+        <f>Data!G11</f>
         <v>0.73199999999999998</v>
       </c>
     </row>
@@ -4969,19 +5033,19 @@
         <v>15</v>
       </c>
       <c r="B11" s="5">
-        <f>nba_team_financials!C12/nba_team_financials!E12</f>
+        <f>Data!C12/Data!E12</f>
         <v>23783783.783783782</v>
       </c>
       <c r="C11" s="6">
-        <f>nba_team_financials!E12/(nba_team_financials!B12/1000000)</f>
+        <f>Data!E12/(Data!B12/1000000)</f>
         <v>0.1579693003742485</v>
       </c>
       <c r="D11" s="4">
-        <f>nba_team_financials!C12/nba_team_financials!B12</f>
+        <f>Data!C12/Data!B12</f>
         <v>3.7571076845767206</v>
       </c>
       <c r="E11" s="24">
-        <f>nba_team_financials!G12</f>
+        <f>Data!G12</f>
         <v>0.45100000000000001</v>
       </c>
     </row>
@@ -4990,19 +5054,19 @@
         <v>16</v>
       </c>
       <c r="B12" s="5">
-        <f>nba_team_financials!C13/nba_team_financials!E13</f>
+        <f>Data!C13/Data!E13</f>
         <v>8980769.2307692301</v>
       </c>
       <c r="C12" s="6">
-        <f>nba_team_financials!E13/(nba_team_financials!B13/1000000)</f>
+        <f>Data!E13/(Data!B13/1000000)</f>
         <v>0.2581766480770874</v>
       </c>
       <c r="D12" s="4">
-        <f>nba_team_financials!C13/nba_team_financials!B13</f>
+        <f>Data!C13/Data!B13</f>
         <v>2.3186248971538426</v>
       </c>
       <c r="E12" s="24">
-        <f>nba_team_financials!G13</f>
+        <f>Data!G13</f>
         <v>0.63400000000000001</v>
       </c>
     </row>
@@ -5011,19 +5075,19 @@
         <v>17</v>
       </c>
       <c r="B13" s="5">
-        <f>nba_team_financials!C14/nba_team_financials!E14</f>
+        <f>Data!C14/Data!E14</f>
         <v>18000000</v>
       </c>
       <c r="C13" s="6">
-        <f>nba_team_financials!E14/(nba_team_financials!B14/1000000)</f>
+        <f>Data!E14/(Data!B14/1000000)</f>
         <v>9.9009794189539355E-2</v>
       </c>
       <c r="D13" s="4">
-        <f>nba_team_financials!C14/nba_team_financials!B14</f>
+        <f>Data!C14/Data!B14</f>
         <v>1.7821762954117084</v>
       </c>
       <c r="E13" s="24">
-        <f>nba_team_financials!G14</f>
+        <f>Data!G14</f>
         <v>0.23200000000000001</v>
       </c>
     </row>
@@ -5032,19 +5096,19 @@
         <v>18</v>
       </c>
       <c r="B14" s="5">
-        <f>nba_team_financials!C15/nba_team_financials!E15</f>
+        <f>Data!C15/Data!E15</f>
         <v>13547619.047619049</v>
       </c>
       <c r="C14" s="6">
-        <f>nba_team_financials!E15/(nba_team_financials!B15/1000000)</f>
+        <f>Data!E15/(Data!B15/1000000)</f>
         <v>0.21099777683699564</v>
       </c>
       <c r="D14" s="4">
-        <f>nba_team_financials!C15/nba_team_financials!B15</f>
+        <f>Data!C15/Data!B15</f>
         <v>2.8585175004821552</v>
       </c>
       <c r="E14" s="24">
-        <f>nba_team_financials!G15</f>
+        <f>Data!G15</f>
         <v>0.51200000000000001</v>
       </c>
     </row>
@@ -5053,19 +5117,19 @@
         <v>19</v>
       </c>
       <c r="B15" s="5">
-        <f>nba_team_financials!C16/nba_team_financials!E16</f>
+        <f>Data!C16/Data!E16</f>
         <v>10396226.41509434</v>
       </c>
       <c r="C15" s="6">
-        <f>nba_team_financials!E16/(nba_team_financials!B16/1000000)</f>
+        <f>Data!E16/(Data!B16/1000000)</f>
         <v>0.25071015187893281</v>
       </c>
       <c r="D15" s="4">
-        <f>nba_team_financials!C16/nba_team_financials!B16</f>
+        <f>Data!C16/Data!B16</f>
         <v>2.606439503496075</v>
       </c>
       <c r="E15" s="24">
-        <f>nba_team_financials!G16</f>
+        <f>Data!G16</f>
         <v>0.64600000000000002</v>
       </c>
     </row>
@@ -5074,19 +5138,19 @@
         <v>20</v>
       </c>
       <c r="B16" s="5">
-        <f>nba_team_financials!C17/nba_team_financials!E17</f>
+        <f>Data!C17/Data!E17</f>
         <v>12240000</v>
       </c>
       <c r="C16" s="6">
-        <f>nba_team_financials!E17/(nba_team_financials!B17/1000000)</f>
+        <f>Data!E17/(Data!B17/1000000)</f>
         <v>0.15857884430719552</v>
       </c>
       <c r="D16" s="4">
-        <f>nba_team_financials!C17/nba_team_financials!B17</f>
+        <f>Data!C17/Data!B17</f>
         <v>1.941005054320073</v>
       </c>
       <c r="E16" s="24">
-        <f>nba_team_financials!G17</f>
+        <f>Data!G17</f>
         <v>0.30499999999999999</v>
       </c>
     </row>
@@ -5095,19 +5159,19 @@
         <v>21</v>
       </c>
       <c r="B17" s="5">
-        <f>nba_team_financials!C18/nba_team_financials!E18</f>
+        <f>Data!C18/Data!E18</f>
         <v>9697674.4186046515</v>
       </c>
       <c r="C17" s="6">
-        <f>nba_team_financials!E18/(nba_team_financials!B18/1000000)</f>
+        <f>Data!E18/(Data!B18/1000000)</f>
         <v>0.21722430959067249</v>
       </c>
       <c r="D17" s="4">
-        <f>nba_team_financials!C18/nba_team_financials!B18</f>
+        <f>Data!C18/Data!B18</f>
         <v>2.1065706302165217</v>
       </c>
       <c r="E17" s="24">
-        <f>nba_team_financials!G18</f>
+        <f>Data!G18</f>
         <v>0.52400000000000002</v>
       </c>
     </row>
@@ -5116,19 +5180,19 @@
         <v>22</v>
       </c>
       <c r="B18" s="5">
-        <f>nba_team_financials!C19/nba_team_financials!E19</f>
+        <f>Data!C19/Data!E19</f>
         <v>11093750</v>
       </c>
       <c r="C18" s="6">
-        <f>nba_team_financials!E19/(nba_team_financials!B19/1000000)</f>
+        <f>Data!E19/(Data!B19/1000000)</f>
         <v>0.17654647401106252</v>
       </c>
       <c r="D18" s="4">
-        <f>nba_team_financials!C19/nba_team_financials!B19</f>
+        <f>Data!C19/Data!B19</f>
         <v>1.9585624460602247</v>
       </c>
       <c r="E18" s="24">
-        <f>nba_team_financials!G19</f>
+        <f>Data!G19</f>
         <v>0.39</v>
       </c>
     </row>
@@ -5137,19 +5201,19 @@
         <v>23</v>
       </c>
       <c r="B19" s="5">
-        <f>nba_team_financials!C20/nba_team_financials!E20</f>
+        <f>Data!C20/Data!E20</f>
         <v>6530612.2448979588</v>
       </c>
       <c r="C19" s="6">
-        <f>nba_team_financials!E20/(nba_team_financials!B20/1000000)</f>
+        <f>Data!E20/(Data!B20/1000000)</f>
         <v>0.21412219141547689</v>
       </c>
       <c r="D19" s="4">
-        <f>nba_team_financials!C20/nba_team_financials!B20</f>
+        <f>Data!C20/Data!B20</f>
         <v>1.3983490051622982</v>
       </c>
       <c r="E19" s="24">
-        <f>nba_team_financials!G20</f>
+        <f>Data!G20</f>
         <v>0.59799999999999998</v>
       </c>
     </row>
@@ -5158,19 +5222,19 @@
         <v>24</v>
       </c>
       <c r="B20" s="5">
-        <f>nba_team_financials!C21/nba_team_financials!E21</f>
+        <f>Data!C21/Data!E21</f>
         <v>11615384.615384616</v>
       </c>
       <c r="C20" s="6">
-        <f>nba_team_financials!E21/(nba_team_financials!B21/1000000)</f>
+        <f>Data!E21/(Data!B21/1000000)</f>
         <v>0.12532942719428955</v>
       </c>
       <c r="D20" s="4">
-        <f>nba_team_financials!C21/nba_team_financials!B21</f>
+        <f>Data!C21/Data!B21</f>
         <v>1.4557495004875169</v>
       </c>
       <c r="E20" s="24">
-        <f>nba_team_financials!G21</f>
+        <f>Data!G21</f>
         <v>0.317</v>
       </c>
     </row>
@@ -5179,19 +5243,19 @@
         <v>25</v>
       </c>
       <c r="B21" s="5">
-        <f>nba_team_financials!C22/nba_team_financials!E22</f>
+        <f>Data!C22/Data!E22</f>
         <v>10037735.849056603</v>
       </c>
       <c r="C21" s="6">
-        <f>nba_team_financials!E22/(nba_team_financials!B22/1000000)</f>
+        <f>Data!E22/(Data!B22/1000000)</f>
         <v>0.25268111588824627</v>
       </c>
       <c r="D21" s="4">
-        <f>nba_team_financials!C22/nba_team_financials!B22</f>
+        <f>Data!C22/Data!B22</f>
         <v>2.5363462953310756</v>
       </c>
       <c r="E21" s="24">
-        <f>nba_team_financials!G22</f>
+        <f>Data!G22</f>
         <v>0.64600000000000002</v>
       </c>
     </row>
@@ -5200,19 +5264,19 @@
         <v>26</v>
       </c>
       <c r="B22" s="5">
-        <f>nba_team_financials!C23/nba_team_financials!E23</f>
+        <f>Data!C23/Data!E23</f>
         <v>5578125</v>
       </c>
       <c r="C22" s="6">
-        <f>nba_team_financials!E23/(nba_team_financials!B23/1000000)</f>
+        <f>Data!E23/(Data!B23/1000000)</f>
         <v>0.34032079818925087</v>
       </c>
       <c r="D22" s="4">
-        <f>nba_team_financials!C23/nba_team_financials!B23</f>
+        <f>Data!C23/Data!B23</f>
         <v>1.898351952399415</v>
       </c>
       <c r="E22" s="24">
-        <f>nba_team_financials!G23</f>
+        <f>Data!G23</f>
         <v>0.78</v>
       </c>
     </row>
@@ -5221,19 +5285,19 @@
         <v>27</v>
       </c>
       <c r="B23" s="5">
-        <f>nba_team_financials!C24/nba_team_financials!E24</f>
+        <f>Data!C24/Data!E24</f>
         <v>7066666.666666667</v>
       </c>
       <c r="C23" s="6">
-        <f>nba_team_financials!E24/(nba_team_financials!B24/1000000)</f>
+        <f>Data!E24/(Data!B24/1000000)</f>
         <v>0.23188272686707773</v>
       </c>
       <c r="D23" s="4">
-        <f>nba_team_financials!C24/nba_team_financials!B24</f>
+        <f>Data!C24/Data!B24</f>
         <v>1.6386379365273491</v>
       </c>
       <c r="E23" s="24">
-        <f>nba_team_financials!G24</f>
+        <f>Data!G24</f>
         <v>0.54900000000000004</v>
       </c>
     </row>
@@ -5242,19 +5306,19 @@
         <v>28</v>
       </c>
       <c r="B24" s="5">
-        <f>nba_team_financials!C25/nba_team_financials!E25</f>
+        <f>Data!C25/Data!E25</f>
         <v>10488888.888888888</v>
       </c>
       <c r="C24" s="6">
-        <f>nba_team_financials!E25/(nba_team_financials!B25/1000000)</f>
+        <f>Data!E25/(Data!B25/1000000)</f>
         <v>0.22511432318345712</v>
       </c>
       <c r="D24" s="4">
-        <f>nba_team_financials!C25/nba_team_financials!B25</f>
+        <f>Data!C25/Data!B25</f>
         <v>2.3611991231687055</v>
       </c>
       <c r="E24" s="24">
-        <f>nba_team_financials!G25</f>
+        <f>Data!G25</f>
         <v>0.54900000000000004</v>
       </c>
     </row>
@@ -5263,19 +5327,19 @@
         <v>29</v>
       </c>
       <c r="B25" s="5">
-        <f>nba_team_financials!C26/nba_team_financials!E26</f>
+        <f>Data!C26/Data!E26</f>
         <v>10111111.111111112</v>
       </c>
       <c r="C25" s="6">
-        <f>nba_team_financials!E26/(nba_team_financials!B26/1000000)</f>
+        <f>Data!E26/(Data!B26/1000000)</f>
         <v>0.2165575171062753</v>
       </c>
       <c r="D25" s="4">
-        <f>nba_team_financials!C26/nba_team_financials!B26</f>
+        <f>Data!C26/Data!B26</f>
         <v>2.1896371174078948</v>
       </c>
       <c r="E25" s="24">
-        <f>nba_team_financials!G26</f>
+        <f>Data!G26</f>
         <v>0.54900000000000004</v>
       </c>
     </row>
@@ -5284,19 +5348,19 @@
         <v>30</v>
       </c>
       <c r="B26" s="5">
-        <f>nba_team_financials!C27/nba_team_financials!E27</f>
+        <f>Data!C27/Data!E27</f>
         <v>8595238.0952380951</v>
       </c>
       <c r="C26" s="6">
-        <f>nba_team_financials!E27/(nba_team_financials!B27/1000000)</f>
+        <f>Data!E27/(Data!B27/1000000)</f>
         <v>0.21219856600048881</v>
       </c>
       <c r="D26" s="4">
-        <f>nba_team_financials!C27/nba_team_financials!B27</f>
+        <f>Data!C27/Data!B27</f>
         <v>1.8238971982422967</v>
       </c>
       <c r="E26" s="24">
-        <f>nba_team_financials!G27</f>
+        <f>Data!G27</f>
         <v>0.51200000000000001</v>
       </c>
     </row>
@@ -5305,19 +5369,19 @@
         <v>31</v>
       </c>
       <c r="B27" s="5">
-        <f>nba_team_financials!C28/nba_team_financials!E28</f>
+        <f>Data!C28/Data!E28</f>
         <v>16090909.090909092</v>
       </c>
       <c r="C27" s="6">
-        <f>nba_team_financials!E28/(nba_team_financials!B28/1000000)</f>
+        <f>Data!E28/(Data!B28/1000000)</f>
         <v>0.10287422687271296</v>
       </c>
       <c r="D27" s="4">
-        <f>nba_team_financials!C28/nba_team_financials!B28</f>
+        <f>Data!C28/Data!B28</f>
         <v>1.6553398324063813</v>
       </c>
       <c r="E27" s="24">
-        <f>nba_team_financials!G28</f>
+        <f>Data!G28</f>
         <v>0.26800000000000002</v>
       </c>
     </row>
@@ -5326,19 +5390,19 @@
         <v>32</v>
       </c>
       <c r="B28" s="5">
-        <f>nba_team_financials!C29/nba_team_financials!E29</f>
+        <f>Data!C29/Data!E29</f>
         <v>6467741.935483871</v>
       </c>
       <c r="C28" s="6">
-        <f>nba_team_financials!E29/(nba_team_financials!B29/1000000)</f>
+        <f>Data!E29/(Data!B29/1000000)</f>
         <v>0.33697361033020645</v>
       </c>
       <c r="D28" s="4">
-        <f>nba_team_financials!C29/nba_team_financials!B29</f>
+        <f>Data!C29/Data!B29</f>
         <v>2.1794583506840772</v>
       </c>
       <c r="E28" s="24">
-        <f>nba_team_financials!G29</f>
+        <f>Data!G29</f>
         <v>0.75600000000000001</v>
       </c>
     </row>
@@ -5347,19 +5411,19 @@
         <v>33</v>
       </c>
       <c r="B29" s="5">
-        <f>nba_team_financials!C30/nba_team_financials!E30</f>
+        <f>Data!C30/Data!E30</f>
         <v>8260869.5652173916</v>
       </c>
       <c r="C29" s="6">
-        <f>nba_team_financials!E30/(nba_team_financials!B30/1000000)</f>
+        <f>Data!E30/(Data!B30/1000000)</f>
         <v>0.23593854970214811</v>
       </c>
       <c r="D29" s="4">
-        <f>nba_team_financials!C30/nba_team_financials!B30</f>
+        <f>Data!C30/Data!B30</f>
         <v>1.9490575844960061</v>
       </c>
       <c r="E29" s="24">
-        <f>nba_team_financials!G30</f>
+        <f>Data!G30</f>
         <v>0.56100000000000005</v>
       </c>
     </row>
@@ -5368,19 +5432,19 @@
         <v>34</v>
       </c>
       <c r="B30" s="5">
-        <f>nba_team_financials!C31/nba_team_financials!E31</f>
+        <f>Data!C31/Data!E31</f>
         <v>15454545.454545455</v>
       </c>
       <c r="C30" s="6">
-        <f>nba_team_financials!E31/(nba_team_financials!B31/1000000)</f>
+        <f>Data!E31/(Data!B31/1000000)</f>
         <v>0.12708143285216664</v>
       </c>
       <c r="D30" s="4">
-        <f>nba_team_financials!C31/nba_team_financials!B31</f>
+        <f>Data!C31/Data!B31</f>
         <v>1.9639857804425753</v>
       </c>
       <c r="E30" s="24">
-        <f>nba_team_financials!G31</f>
+        <f>Data!G31</f>
         <v>0.26800000000000002</v>
       </c>
     </row>
@@ -5389,19 +5453,19 @@
         <v>35</v>
       </c>
       <c r="B31" s="5">
-        <f>nba_team_financials!C32/nba_team_financials!E32</f>
+        <f>Data!C32/Data!E32</f>
         <v>22882352.94117647</v>
       </c>
       <c r="C31" s="6">
-        <f>nba_team_financials!E32/(nba_team_financials!B32/1000000)</f>
+        <f>Data!E32/(Data!B32/1000000)</f>
         <v>7.3265315337343442E-2</v>
       </c>
       <c r="D31" s="4">
-        <f>nba_team_financials!C32/nba_team_financials!B32</f>
+        <f>Data!C32/Data!B32</f>
         <v>1.6764828038956823</v>
       </c>
       <c r="E31" s="24">
-        <f>nba_team_financials!G32</f>
+        <f>Data!G32</f>
         <v>0.20699999999999999</v>
       </c>
     </row>
@@ -5412,25 +5476,25 @@
       <c r="A33" s="17"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A34" s="57" t="s">
+      <c r="A34" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="B34" s="58" t="s">
+      <c r="B34" s="55" t="s">
         <v>55</v>
       </c>
-      <c r="C34" s="58" t="s">
+      <c r="C34" s="55" t="s">
         <v>56</v>
       </c>
-      <c r="D34" s="58" t="s">
+      <c r="D34" s="55" t="s">
         <v>57</v>
       </c>
-      <c r="E34" s="58" t="s">
+      <c r="E34" s="55" t="s">
         <v>62</v>
       </c>
-      <c r="F34" s="58" t="s">
+      <c r="F34" s="55" t="s">
         <v>58</v>
       </c>
-      <c r="G34" s="59" t="s">
+      <c r="G34" s="56" t="s">
         <v>59</v>
       </c>
     </row>
@@ -6368,45 +6432,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="48" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="51" t="s">
+      <c r="B1" s="48" t="s">
         <v>58</v>
       </c>
-      <c r="C1" s="51" t="s">
+      <c r="C1" s="48" t="s">
         <v>59</v>
       </c>
-      <c r="D1" s="52" t="s">
+      <c r="D1" s="49" t="s">
         <v>62</v>
       </c>
-      <c r="F1" s="47" t="s">
+      <c r="F1" s="44" t="s">
         <v>47</v>
       </c>
-      <c r="G1" s="47" t="s">
+      <c r="G1" s="44" t="s">
         <v>48</v>
       </c>
-      <c r="H1" s="47" t="s">
+      <c r="H1" s="44" t="s">
         <v>54</v>
       </c>
-      <c r="I1" s="47" t="s">
+      <c r="I1" s="44" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="54" t="str">
+      <c r="A2" s="51" t="str">
         <f xml:space="preserve"> Calculations!A48</f>
         <v>Los Angeles Lakers</v>
       </c>
-      <c r="B2" s="55">
+      <c r="B2" s="52">
         <f>Calculations!F48</f>
         <v>7.1999999999999993</v>
       </c>
-      <c r="C2" s="56">
+      <c r="C2" s="53">
         <f>Calculations!G48</f>
         <v>1</v>
       </c>
-      <c r="D2" s="56">
+      <c r="D2" s="53">
         <f>Calculations!E48</f>
         <v>6</v>
       </c>
@@ -6428,7 +6492,7 @@
         <f xml:space="preserve"> Calculations!A54</f>
         <v>New York Knicks</v>
       </c>
-      <c r="B3" s="53">
+      <c r="B3" s="50">
         <f>Calculations!F54</f>
         <v>7.65</v>
       </c>
@@ -6458,7 +6522,7 @@
         <f xml:space="preserve"> Calculations!A36</f>
         <v>Boston Celtics</v>
       </c>
-      <c r="B4" s="53">
+      <c r="B4" s="50">
         <f>Calculations!F36</f>
         <v>8.0499999999999989</v>
       </c>
@@ -6488,7 +6552,7 @@
         <f xml:space="preserve"> Calculations!A61</f>
         <v>San Antonio Spurs</v>
       </c>
-      <c r="B5" s="53">
+      <c r="B5" s="50">
         <f>Calculations!F61</f>
         <v>8.8999999999999986</v>
       </c>
@@ -6518,7 +6582,7 @@
         <f xml:space="preserve"> Calculations!A45</f>
         <v>Houston Rockets</v>
       </c>
-      <c r="B6" s="53">
+      <c r="B6" s="50">
         <f>Calculations!F45</f>
         <v>9.35</v>
       </c>
@@ -6548,7 +6612,7 @@
         <f xml:space="preserve"> Calculations!A35</f>
         <v>Atlanta Hawks</v>
       </c>
-      <c r="B7" s="53">
+      <c r="B7" s="50">
         <f>Calculations!F35</f>
         <v>9.8000000000000007</v>
       </c>
@@ -6578,7 +6642,7 @@
         <f xml:space="preserve"> Calculations!A55</f>
         <v>Oklahoma City Thunder</v>
       </c>
-      <c r="B8" s="53">
+      <c r="B8" s="50">
         <f>Calculations!F55</f>
         <v>10.899999999999999</v>
       </c>
@@ -6596,7 +6660,7 @@
         <f xml:space="preserve"> Calculations!A57</f>
         <v>Philadelphia 76ers</v>
       </c>
-      <c r="B9" s="53">
+      <c r="B9" s="50">
         <f>Calculations!F57</f>
         <v>11.5</v>
       </c>
@@ -6614,7 +6678,7 @@
         <f xml:space="preserve"> Calculations!A47</f>
         <v>Los Angeles Clippers</v>
       </c>
-      <c r="B10" s="53">
+      <c r="B10" s="50">
         <f>Calculations!F47</f>
         <v>12.149999999999999</v>
       </c>
@@ -6632,7 +6696,7 @@
         <f xml:space="preserve"> Calculations!A44</f>
         <v>Golden State Warriors</v>
       </c>
-      <c r="B11" s="53">
+      <c r="B11" s="50">
         <f>Calculations!F44</f>
         <v>12.35</v>
       </c>
@@ -6650,7 +6714,7 @@
         <f xml:space="preserve"> Calculations!A42</f>
         <v>Denver Nuggets</v>
       </c>
-      <c r="B12" s="53">
+      <c r="B12" s="50">
         <f>Calculations!F42</f>
         <v>13.25</v>
       </c>
@@ -6668,7 +6732,7 @@
         <f xml:space="preserve"> Calculations!A58</f>
         <v>Phoenix Suns</v>
       </c>
-      <c r="B13" s="53">
+      <c r="B13" s="50">
         <f>Calculations!F58</f>
         <v>13.75</v>
       </c>
@@ -6686,7 +6750,7 @@
         <f xml:space="preserve"> Calculations!A43</f>
         <v>Detroit Pistons</v>
       </c>
-      <c r="B14" s="53">
+      <c r="B14" s="50">
         <f>Calculations!F43</f>
         <v>13.95</v>
       </c>
@@ -6704,7 +6768,7 @@
         <f xml:space="preserve"> Calculations!A62</f>
         <v>Toronto Raptors</v>
       </c>
-      <c r="B15" s="53">
+      <c r="B15" s="50">
         <f>Calculations!F62</f>
         <v>14.45</v>
       </c>
@@ -6722,7 +6786,7 @@
         <f xml:space="preserve"> Calculations!A40</f>
         <v>Cleveland Cavaliers</v>
       </c>
-      <c r="B16" s="53">
+      <c r="B16" s="50">
         <f>Calculations!F40</f>
         <v>14.45</v>
       </c>
@@ -6740,7 +6804,7 @@
         <f xml:space="preserve"> Calculations!A50</f>
         <v>Miami Heat</v>
       </c>
-      <c r="B17" s="53">
+      <c r="B17" s="50">
         <f>Calculations!F50</f>
         <v>15.35</v>
       </c>
@@ -6758,7 +6822,7 @@
         <f xml:space="preserve"> Calculations!A37</f>
         <v>Brooklyn Nets</v>
       </c>
-      <c r="B18" s="53">
+      <c r="B18" s="50">
         <f>Calculations!F37</f>
         <v>15.549999999999999</v>
       </c>
@@ -6776,7 +6840,7 @@
         <f xml:space="preserve"> Calculations!A39</f>
         <v>Chicago Bulls</v>
       </c>
-      <c r="B19" s="53">
+      <c r="B19" s="50">
         <f>Calculations!F39</f>
         <v>16</v>
       </c>
@@ -6794,7 +6858,7 @@
         <f xml:space="preserve"> Calculations!A38</f>
         <v>Charlotte Hornets</v>
       </c>
-      <c r="B20" s="53">
+      <c r="B20" s="50">
         <f>Calculations!F38</f>
         <v>17.2</v>
       </c>
@@ -6812,7 +6876,7 @@
         <f xml:space="preserve"> Calculations!A51</f>
         <v>Milwaukee Bucks</v>
       </c>
-      <c r="B21" s="53">
+      <c r="B21" s="50">
         <f>Calculations!F51</f>
         <v>17.850000000000001</v>
       </c>
@@ -6830,7 +6894,7 @@
         <f xml:space="preserve"> Calculations!A41</f>
         <v>Dallas Mavericks</v>
       </c>
-      <c r="B22" s="53">
+      <c r="B22" s="50">
         <f>Calculations!F41</f>
         <v>18.350000000000001</v>
       </c>
@@ -6848,7 +6912,7 @@
         <f xml:space="preserve"> Calculations!A56</f>
         <v>Orlando Magic</v>
       </c>
-      <c r="B23" s="53">
+      <c r="B23" s="50">
         <f>Calculations!F56</f>
         <v>19</v>
       </c>
@@ -6866,7 +6930,7 @@
         <f xml:space="preserve"> Calculations!A59</f>
         <v>Portland Trail Blazers</v>
       </c>
-      <c r="B24" s="53">
+      <c r="B24" s="50">
         <f>Calculations!F59</f>
         <v>19.2</v>
       </c>
@@ -6884,7 +6948,7 @@
         <f xml:space="preserve"> Calculations!A63</f>
         <v>Utah Jazz</v>
       </c>
-      <c r="B25" s="53">
+      <c r="B25" s="50">
         <f>Calculations!F63</f>
         <v>19.850000000000001</v>
       </c>
@@ -6902,7 +6966,7 @@
         <f xml:space="preserve"> Calculations!A49</f>
         <v>Memphis Grizzlies</v>
       </c>
-      <c r="B26" s="53">
+      <c r="B26" s="50">
         <f>Calculations!F49</f>
         <v>20.05</v>
       </c>
@@ -6920,7 +6984,7 @@
         <f xml:space="preserve"> Calculations!A52</f>
         <v>Minnesota Timberwolves</v>
       </c>
-      <c r="B27" s="53">
+      <c r="B27" s="50">
         <f>Calculations!F52</f>
         <v>20.65</v>
       </c>
@@ -6938,7 +7002,7 @@
         <f xml:space="preserve"> Calculations!A46</f>
         <v>Indiana Pacers</v>
       </c>
-      <c r="B28" s="53">
+      <c r="B28" s="50">
         <f>Calculations!F46</f>
         <v>23.75</v>
       </c>
@@ -6956,7 +7020,7 @@
         <f xml:space="preserve"> Calculations!A60</f>
         <v>Sacramento Kings</v>
       </c>
-      <c r="B29" s="53">
+      <c r="B29" s="50">
         <f>Calculations!F60</f>
         <v>23.75</v>
       </c>
@@ -6974,7 +7038,7 @@
         <f xml:space="preserve"> Calculations!A53</f>
         <v>New Orleans Pelicans</v>
       </c>
-      <c r="B30" s="53">
+      <c r="B30" s="50">
         <f>Calculations!F53</f>
         <v>24.199999999999996</v>
       </c>
@@ -6992,7 +7056,7 @@
         <f xml:space="preserve"> Calculations!A64</f>
         <v>Washington Wizards</v>
       </c>
-      <c r="B31" s="53">
+      <c r="B31" s="50">
         <f>Calculations!F64</f>
         <v>24.3</v>
       </c>
@@ -7019,7 +7083,7 @@
   <sheetPr>
     <tabColor rgb="FF1F4E79"/>
   </sheetPr>
-  <dimension ref="A1:T12"/>
+  <dimension ref="A1:R14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15" style="3" customWidth="1"/>
@@ -7035,352 +7099,355 @@
     <col min="15" max="16384" width="10.83203125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="60" t="s">
+    <row r="1" spans="1:18" ht="21" x14ac:dyDescent="0.25">
+      <c r="A1" s="61" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-    </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B2" s="43" t="s">
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+    </row>
+    <row r="2" spans="1:18" ht="21" x14ac:dyDescent="0.25">
+      <c r="A2" s="57"/>
+      <c r="B2" s="60" t="s">
+        <v>95</v>
+      </c>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="58"/>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B4" s="40" t="s">
         <v>73</v>
       </c>
-      <c r="C2" s="44"/>
-      <c r="D2" s="45"/>
-      <c r="F2" s="43" t="s">
+      <c r="C4" s="41"/>
+      <c r="D4" s="42"/>
+      <c r="F4" s="40" t="s">
         <v>74</v>
       </c>
-      <c r="G2" s="44"/>
-      <c r="H2" s="45"/>
-      <c r="J2" s="43" t="s">
+      <c r="G4" s="41"/>
+      <c r="H4" s="42"/>
+      <c r="J4" s="40" t="s">
         <v>75</v>
       </c>
-      <c r="K2" s="44"/>
-      <c r="L2" s="45"/>
-      <c r="N2" s="43" t="s">
+      <c r="K4" s="41"/>
+      <c r="L4" s="42"/>
+      <c r="N4" s="59" t="s">
         <v>76</v>
       </c>
-      <c r="O2" s="44"/>
-      <c r="P2" s="45"/>
-      <c r="R2" s="46" t="s">
+      <c r="P4" s="43" t="s">
         <v>77</v>
       </c>
-      <c r="S2" s="46"/>
-      <c r="T2" s="46"/>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B3" s="28" t="str">
+      <c r="Q4" s="43"/>
+      <c r="R4" s="43"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B5" s="28" t="str">
         <f>Rankings!A2</f>
         <v>Los Angeles Lakers</v>
       </c>
-      <c r="C3" s="29"/>
-      <c r="D3" s="30"/>
-      <c r="F3" s="28" t="str">
+      <c r="C5" s="29"/>
+      <c r="D5" s="30"/>
+      <c r="F5" s="28" t="str">
         <f>INDEX(Calculations!$A$35:$A$64,MATCH(1,Calculations!$C$35:$C$64,0))</f>
         <v>Oklahoma City Thunder</v>
       </c>
-      <c r="G3" s="29"/>
-      <c r="H3" s="30"/>
-      <c r="J3" s="28" t="str">
+      <c r="G5" s="29"/>
+      <c r="H5" s="30"/>
+      <c r="J5" s="28" t="str">
         <f>INDEX(Calculations!$A$35:$A$64,MATCH(1,Calculations!$D$35:$D$64,0))</f>
         <v>Golden State Warriors</v>
       </c>
-      <c r="K3" s="29"/>
-      <c r="L3" s="30"/>
-      <c r="N3" s="28" t="str">
+      <c r="K5" s="29"/>
+      <c r="L5" s="30"/>
+      <c r="N5" s="28" t="str">
         <f>INDEX(Calculations!$A$2:$A$31,MATCH(MAX(Calculations!$E$2:$E$31),Calculations!$E$2:$E$31,0))</f>
         <v>Oklahoma City Thunder</v>
       </c>
-      <c r="O3" s="29"/>
-      <c r="P3" s="30"/>
-      <c r="R3" s="37">
-        <f>AVERAGE(nba_team_financials!$B$3:$B$32)/1000000</f>
+      <c r="P5" s="34">
+        <f>AVERAGE(Data!$B$3:$B$32)/1000000</f>
         <v>197.90667206666666</v>
       </c>
-      <c r="S3" s="38"/>
-      <c r="T3" s="39"/>
-    </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B4" s="31"/>
-      <c r="C4" s="32"/>
-      <c r="D4" s="33"/>
-      <c r="F4" s="31"/>
-      <c r="G4" s="32"/>
-      <c r="H4" s="33"/>
-      <c r="J4" s="31"/>
-      <c r="K4" s="32"/>
-      <c r="L4" s="33"/>
-      <c r="N4" s="31"/>
-      <c r="O4" s="32"/>
-      <c r="P4" s="33"/>
-      <c r="R4" s="40"/>
-      <c r="S4" s="41"/>
-      <c r="T4" s="42"/>
-    </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="N5" s="34">
+      <c r="Q5" s="35"/>
+      <c r="R5" s="36"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B6" s="31"/>
+      <c r="C6" s="32"/>
+      <c r="D6" s="33"/>
+      <c r="F6" s="31"/>
+      <c r="G6" s="32"/>
+      <c r="H6" s="33"/>
+      <c r="J6" s="31"/>
+      <c r="K6" s="32"/>
+      <c r="L6" s="33"/>
+      <c r="N6" s="31"/>
+      <c r="P6" s="37"/>
+      <c r="Q6" s="38"/>
+      <c r="R6" s="39"/>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="N7" s="62">
         <f>MAX(Calculations!$E$2:$E$31)</f>
         <v>0.78</v>
       </c>
-      <c r="O5" s="35"/>
-      <c r="P5" s="36"/>
-    </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B6" s="25" t="s">
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B8" s="25" t="s">
         <v>81</v>
       </c>
-      <c r="C6" s="25"/>
-      <c r="D6" s="25"/>
-      <c r="E6" s="25"/>
-      <c r="J6" s="25" t="s">
+      <c r="C8" s="25"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="25"/>
+      <c r="J8" s="25" t="s">
         <v>82</v>
       </c>
-      <c r="K6" s="25"/>
-      <c r="L6" s="25"/>
-      <c r="M6" s="25"/>
-    </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B7" s="47" t="s">
+      <c r="K8" s="25"/>
+      <c r="L8" s="25"/>
+      <c r="M8" s="25"/>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B9" s="44" t="s">
         <v>80</v>
       </c>
-      <c r="C7" s="47" t="s">
+      <c r="C9" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="47" t="s">
+      <c r="D9" s="44" t="s">
         <v>58</v>
       </c>
-      <c r="E7" s="47" t="s">
+      <c r="E9" s="44" t="s">
         <v>62</v>
       </c>
-      <c r="F7" s="47" t="s">
+      <c r="F9" s="44" t="s">
         <v>83</v>
       </c>
-      <c r="J7" s="47" t="s">
+      <c r="J9" s="44" t="s">
         <v>80</v>
       </c>
-      <c r="K7" s="47" t="s">
+      <c r="K9" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="L7" s="47" t="s">
+      <c r="L9" s="44" t="s">
         <v>58</v>
       </c>
-      <c r="M7" s="47" t="s">
+      <c r="M9" s="44" t="s">
         <v>62</v>
       </c>
-      <c r="N7" s="47" t="s">
+      <c r="N9" s="44" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="8" spans="1:20" ht="16" x14ac:dyDescent="0.2">
-      <c r="B8" s="3">
+    <row r="10" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C8" s="3" t="str">
+      <c r="C10" s="3" t="str">
         <f>Rankings!A2</f>
         <v>Los Angeles Lakers</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D10" s="3">
         <f>Rankings!B2</f>
         <v>7.1999999999999993</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E10" s="3">
         <f>Rankings!D2</f>
         <v>6</v>
       </c>
-      <c r="F8" s="26" t="s">
+      <c r="F10" s="26" t="s">
         <v>85</v>
       </c>
-      <c r="J8" s="3">
+      <c r="J10" s="3">
         <v>26</v>
       </c>
-      <c r="K8" s="3" t="str">
+      <c r="K10" s="3" t="str">
         <f>Rankings!A27</f>
         <v>Minnesota Timberwolves</v>
       </c>
-      <c r="L8" s="3">
+      <c r="L10" s="3">
         <f>Rankings!B27</f>
         <v>20.65</v>
       </c>
-      <c r="M8" s="3">
+      <c r="M10" s="3">
         <f>Rankings!D27</f>
         <v>10</v>
       </c>
-      <c r="N8" s="27" t="s">
+      <c r="N10" s="27" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B9" s="3">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B11" s="3">
         <v>2</v>
       </c>
-      <c r="C9" s="3" t="str">
+      <c r="C11" s="3" t="str">
         <f>Rankings!A3</f>
         <v>New York Knicks</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D11" s="3">
         <f>Rankings!B3</f>
         <v>7.65</v>
       </c>
-      <c r="E9" s="3">
+      <c r="E11" s="3">
         <f>Rankings!D3</f>
         <v>6</v>
       </c>
-      <c r="F9" s="27" t="s">
+      <c r="F11" s="27" t="s">
         <v>86</v>
       </c>
-      <c r="J9" s="3">
+      <c r="J11" s="3">
         <v>27</v>
       </c>
-      <c r="K9" s="3" t="str">
+      <c r="K11" s="3" t="str">
         <f>Rankings!A28</f>
         <v>Indiana Pacers</v>
       </c>
-      <c r="L9" s="3">
+      <c r="L11" s="3">
         <f>Rankings!B28</f>
         <v>23.75</v>
       </c>
-      <c r="M9" s="3">
+      <c r="M11" s="3">
         <f>Rankings!D28</f>
         <v>29</v>
       </c>
-      <c r="N9" s="27" t="s">
+      <c r="N11" s="27" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B10" s="3">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B12" s="3">
         <v>3</v>
       </c>
-      <c r="C10" s="3" t="str">
+      <c r="C12" s="3" t="str">
         <f>Rankings!A4</f>
         <v>Boston Celtics</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D12" s="3">
         <f>Rankings!B4</f>
         <v>8.0499999999999989</v>
       </c>
-      <c r="E10" s="3">
+      <c r="E12" s="3">
         <f>Rankings!D4</f>
         <v>4</v>
       </c>
-      <c r="F10" s="27" t="s">
+      <c r="F12" s="27" t="s">
         <v>87</v>
       </c>
-      <c r="J10" s="3">
+      <c r="J12" s="3">
         <v>27</v>
       </c>
-      <c r="K10" s="3" t="str">
+      <c r="K12" s="3" t="str">
         <f>Rankings!A29</f>
         <v>Sacramento Kings</v>
       </c>
-      <c r="L10" s="3">
+      <c r="L12" s="3">
         <f>Rankings!B29</f>
         <v>23.75</v>
       </c>
-      <c r="M10" s="3">
+      <c r="M12" s="3">
         <f>Rankings!D29</f>
         <v>26</v>
       </c>
-      <c r="N10" s="27" t="s">
+      <c r="N12" s="27" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B11" s="3">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B13" s="3">
         <v>4</v>
       </c>
-      <c r="C11" s="3" t="str">
+      <c r="C13" s="3" t="str">
         <f>Rankings!A5</f>
         <v>San Antonio Spurs</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D13" s="3">
         <f>Rankings!B5</f>
         <v>8.8999999999999986</v>
       </c>
-      <c r="E11" s="3">
+      <c r="E13" s="3">
         <f>Rankings!D5</f>
         <v>2</v>
       </c>
-      <c r="F11" s="27" t="s">
+      <c r="F13" s="27" t="s">
         <v>88</v>
       </c>
-      <c r="J11" s="3">
+      <c r="J13" s="3">
         <v>29</v>
       </c>
-      <c r="K11" s="3" t="str">
+      <c r="K13" s="3" t="str">
         <f>Rankings!A30</f>
         <v>New Orleans Pelicans</v>
       </c>
-      <c r="L11" s="3">
+      <c r="L13" s="3">
         <f>Rankings!B30</f>
         <v>24.199999999999996</v>
       </c>
-      <c r="M11" s="3">
+      <c r="M13" s="3">
         <f>Rankings!D30</f>
         <v>23</v>
       </c>
-      <c r="N11" s="27" t="s">
+      <c r="N13" s="27" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B12" s="3">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B14" s="3">
         <v>5</v>
       </c>
-      <c r="C12" s="3" t="str">
+      <c r="C14" s="3" t="str">
         <f>Rankings!A6</f>
         <v>Houston Rockets</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D14" s="3">
         <f>Rankings!B6</f>
         <v>9.35</v>
       </c>
-      <c r="E12" s="3">
+      <c r="E14" s="3">
         <f>Rankings!D6</f>
         <v>8</v>
       </c>
-      <c r="F12" s="27" t="s">
+      <c r="F14" s="27" t="s">
         <v>89</v>
       </c>
-      <c r="J12" s="3">
+      <c r="J14" s="3">
         <v>30</v>
       </c>
-      <c r="K12" s="3" t="str">
+      <c r="K14" s="3" t="str">
         <f>Rankings!A31</f>
         <v>Washington Wizards</v>
       </c>
-      <c r="L12" s="3">
+      <c r="L14" s="3">
         <f>Rankings!B31</f>
         <v>24.3</v>
       </c>
-      <c r="M12" s="3">
+      <c r="M14" s="3">
         <f>Rankings!D31</f>
         <v>30</v>
       </c>
-      <c r="N12" s="27" t="s">
+      <c r="N14" s="27" t="s">
         <v>94</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="13">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="N2:P2"/>
-    <mergeCell ref="N3:P4"/>
-    <mergeCell ref="N5:P5"/>
-    <mergeCell ref="R2:T2"/>
-    <mergeCell ref="R3:T4"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="J6:M6"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B3:D4"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="F3:H4"/>
-    <mergeCell ref="J2:L2"/>
-    <mergeCell ref="J3:L4"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="N5:N6"/>
+    <mergeCell ref="P4:R4"/>
+    <mergeCell ref="P5:R6"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="J8:M8"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D6"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="F5:H6"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="J5:L6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
Add updated NBA team financials Excel file
</commit_message>
<xml_diff>
--- a/nba team financials.xlsx
+++ b/nba team financials.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/twandon/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C3DF6C77-F98B-5942-97E6-E86F4F05C915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B1C246CB-3D66-D649-89CF-775B6A5C564A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{060D5569-2AC9-B04F-841D-CEA7829076CD}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17840" activeTab="3" xr2:uid="{060D5569-2AC9-B04F-841D-CEA7829076CD}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -281,9 +281,6 @@
     <t>Wins</t>
   </si>
   <si>
-    <t>NBA Financial &amp; Performance Analysis (2025-26 Season)</t>
-  </si>
-  <si>
     <t>Rank</t>
   </si>
   <si>
@@ -330,6 +327,9 @@
   </si>
   <si>
     <t>Key Question: Does spending more money on players actually make an NBA team win more?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NBA Financial &amp; Performance Analysis (2025-26 Season)			</t>
   </si>
 </sst>
 </file>
@@ -412,12 +412,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color theme="0"/>
@@ -452,6 +446,13 @@
     <font>
       <b/>
       <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -782,79 +783,31 @@
     <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="5" fontId="10" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="5" fontId="11" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -869,38 +822,84 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="10" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="2">
     <dxf>
       <font>
         <b/>
@@ -912,12 +911,6 @@
         <b/>
         <i val="0"/>
         <color rgb="FF1F4E79"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
       </font>
     </dxf>
   </dxfs>
@@ -1388,65 +1381,18 @@
               <c:idx val="0"/>
               <c:tx>
                 <c:rich>
-                  <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-                    <a:spAutoFit/>
-                  </a:bodyPr>
+                  <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:pPr>
-                      <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                        <a:solidFill>
-                          <a:schemeClr val="tx1">
-                            <a:lumMod val="75000"/>
-                            <a:lumOff val="25000"/>
-                          </a:schemeClr>
-                        </a:solidFill>
-                        <a:latin typeface="+mn-lt"/>
-                        <a:ea typeface="+mn-ea"/>
-                        <a:cs typeface="+mn-cs"/>
-                      </a:defRPr>
-                    </a:pPr>
-                    <a:fld id="{0B6D3822-4166-4941-9F10-34006DEAADC7}" type="CELLRANGE">
+                    <a:fld id="{3379A1E9-441E-AA48-82EF-5E4C520726A6}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
-                      <a:pPr>
-                        <a:defRPr/>
-                      </a:pPr>
+                      <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
                     </a:fld>
                     <a:endParaRPr lang="en-US"/>
                   </a:p>
                 </c:rich>
               </c:tx>
-              <c:numFmt formatCode="&quot;$&quot;0.0,,\ &quot;M&quot;" sourceLinked="0"/>
-              <c:spPr>
-                <a:noFill/>
-                <a:ln>
-                  <a:noFill/>
-                </a:ln>
-                <a:effectLst/>
-              </c:spPr>
-              <c:txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-                  <a:spAutoFit/>
-                </a:bodyPr>
-                <a:lstStyle/>
-                <a:p>
-                  <a:pPr>
-                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="75000"/>
-                          <a:lumOff val="25000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:latin typeface="+mn-lt"/>
-                      <a:ea typeface="+mn-ea"/>
-                      <a:cs typeface="+mn-cs"/>
-                    </a:defRPr>
-                  </a:pPr>
-                  <a:endParaRPr lang="en-US"/>
-                </a:p>
-              </c:txPr>
               <c:showLegendKey val="0"/>
               <c:showVal val="0"/>
               <c:showCatName val="0"/>
@@ -1472,7 +1418,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{54AB3A83-D2B2-3249-B332-44BDD9710AF8}" type="CELLRANGE">
+                    <a:fld id="{1F965BF0-0873-DF47-8A48-EF7B8C223EA2}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1512,7 +1458,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{A8E6CECD-2133-2A43-BEBD-52C446C4399C}" type="CELLRANGE">
+                    <a:fld id="{F3963D27-88BF-7745-B2CD-FCE6EF4D5096}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1551,7 +1497,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{99B681EB-D59D-0943-93BA-9408FEE7355B}" type="CELLRANGE">
+                    <a:fld id="{D219E6B1-2CB1-F04F-B5D1-62E9ABEF5072}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1584,7 +1530,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{F2EA1EE5-581B-BE47-AEDA-CCF39245E42E}" type="CELLRANGE">
+                    <a:fld id="{19F2D5E2-FE3B-1E45-B675-F357E448D626}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -3251,15 +3197,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>762001</xdr:colOff>
+      <xdr:colOff>685799</xdr:colOff>
       <xdr:row>32</xdr:row>
-      <xdr:rowOff>118534</xdr:rowOff>
+      <xdr:rowOff>99888</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>42</xdr:row>
-      <xdr:rowOff>84667</xdr:rowOff>
+      <xdr:colOff>156966</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>114158</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -3274,8 +3220,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="762001" y="5723467"/>
-          <a:ext cx="16967200" cy="1828800"/>
+          <a:off x="685799" y="6221573"/>
+          <a:ext cx="15795661" cy="3353372"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3327,7 +3273,7 @@
             <a:defRPr/>
           </a:pPr>
           <a:r>
-            <a:rPr lang="en-US" sz="1050" b="1" i="0">
+            <a:rPr lang="en-US" sz="1250" b="1" i="0">
               <a:solidFill>
                 <a:schemeClr val="dk1"/>
               </a:solidFill>
@@ -3341,7 +3287,7 @@
         </a:p>
         <a:p>
           <a:r>
-            <a:rPr lang="en-US" sz="1050" b="1" i="0">
+            <a:rPr lang="en-US" sz="1250" b="1" i="0">
               <a:solidFill>
                 <a:schemeClr val="dk1"/>
               </a:solidFill>
@@ -3353,7 +3299,7 @@
             <a:t>1. </a:t>
           </a:r>
           <a:r>
-            <a:rPr lang="en-US" sz="1050" b="1" i="0" u="none" strike="noStrike">
+            <a:rPr lang="en-US" sz="1250" b="1" i="0" u="none" strike="noStrike">
               <a:solidFill>
                 <a:schemeClr val="dk1"/>
               </a:solidFill>
@@ -3367,7 +3313,7 @@
         </a:p>
         <a:p>
           <a:r>
-            <a:rPr lang="en-US" sz="1050" b="0" i="0" u="none" strike="noStrike">
+            <a:rPr lang="en-US" sz="1250" b="0" i="0" u="none" strike="noStrike">
               <a:solidFill>
                 <a:schemeClr val="dk1"/>
               </a:solidFill>
@@ -3378,7 +3324,7 @@
             </a:rPr>
             <a:t>Golden State ranked #1 in Revenue-to-Payroll, generating $3.76 in revenue for every $1 of payroll. The Warriors generated $880M in revenue while carrying the NBA's highest payroll at $234.2M. Despite that financial strength, they finished 37–45 with a 45.1% win percentage. The result shows that strong revenue generation does not necessarily translate into competitive success.</a:t>
           </a:r>
-          <a:endParaRPr lang="en-US" sz="1050" b="0" i="0">
+          <a:endParaRPr lang="en-US" sz="1250" b="0" i="0">
             <a:solidFill>
               <a:schemeClr val="dk1"/>
             </a:solidFill>
@@ -3389,7 +3335,7 @@
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:endParaRPr lang="en-US" sz="1050" b="0" i="0">
+          <a:endParaRPr lang="en-US" sz="1250" b="0" i="0">
             <a:solidFill>
               <a:schemeClr val="dk1"/>
             </a:solidFill>
@@ -3401,7 +3347,7 @@
         </a:p>
         <a:p>
           <a:r>
-            <a:rPr lang="en-US" sz="1050" b="1" i="0">
+            <a:rPr lang="en-US" sz="1250" b="1" i="0">
               <a:solidFill>
                 <a:schemeClr val="dk1"/>
               </a:solidFill>
@@ -3413,7 +3359,7 @@
             <a:t>2. </a:t>
           </a:r>
           <a:r>
-            <a:rPr lang="en-US" sz="1050" b="1" i="0" u="none" strike="noStrike">
+            <a:rPr lang="en-US" sz="1250" b="1" i="0" u="none" strike="noStrike">
               <a:solidFill>
                 <a:schemeClr val="dk1"/>
               </a:solidFill>
@@ -3427,18 +3373,20 @@
         </a:p>
         <a:p>
           <a:r>
-            <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:rPr lang="en-US" sz="1250" b="0" i="0" u="none" strike="noStrike">
               <a:solidFill>
                 <a:schemeClr val="dk1"/>
               </a:solidFill>
               <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
               <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
             </a:rPr>
             <a:t>Washington ranked #2 in payroll at $232.0M but finished 30th overall with a 17–65 record. In contrast, San Antonio spent $184.0M, ranked 25th in payroll, and finished 4th overall with 62 wins. The comparison highlights the gap between total spending and spending efficiency. Across all 30 teams, payroll showed only a weak statistical relationship with wins (correlation ≈ 0.17), confirming this pattern holds league-wide, not just in isolated cases.</a:t>
           </a:r>
-          <a:endParaRPr lang="en-US" sz="1050" b="0" i="0">
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-US" sz="1250" b="0" i="0">
             <a:solidFill>
               <a:schemeClr val="dk1"/>
             </a:solidFill>
@@ -3450,7 +3398,7 @@
         </a:p>
         <a:p>
           <a:r>
-            <a:rPr lang="en-US" sz="1050" b="1" i="0">
+            <a:rPr lang="en-US" sz="1250" b="1" i="0">
               <a:solidFill>
                 <a:schemeClr val="dk1"/>
               </a:solidFill>
@@ -3462,7 +3410,7 @@
             <a:t>3. </a:t>
           </a:r>
           <a:r>
-            <a:rPr lang="en-US" sz="1050" b="1" i="0" u="none" strike="noStrike">
+            <a:rPr lang="en-US" sz="1250" b="1" i="0" u="none" strike="noStrike">
               <a:solidFill>
                 <a:schemeClr val="dk1"/>
               </a:solidFill>
@@ -3476,7 +3424,7 @@
         </a:p>
         <a:p>
           <a:r>
-            <a:rPr lang="en-US" sz="1050" b="0" i="0" u="none" strike="noStrike">
+            <a:rPr lang="en-US" sz="1250" b="0" i="0" u="none" strike="noStrike">
               <a:solidFill>
                 <a:schemeClr val="dk1"/>
               </a:solidFill>
@@ -3487,7 +3435,71 @@
             </a:rPr>
             <a:t>Oklahoma City ranked #1 in Win % at 78.0% and #1 in Wins per $1M Payroll at 0.340. The Thunder won 64 games while maintaining a relatively modest $188.1M payroll. Their results represent the strongest combination of competitive performance and payroll efficiency in the dataset.</a:t>
           </a:r>
-          <a:endParaRPr lang="en-US" sz="1050" b="0" i="0">
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-US" sz="1250" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="dk1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1250" b="1" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>Key</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1250" b="1" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t> Takeaway</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1250" b="0" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>The analysis shows that financial resources alone did not determine on-court success. Teams such as Oklahoma City combined strong winning performance with efficient payroll deployment, while teams such as Washington spent heavily without achieving comparable results.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-US" sz="1250" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="dk1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-US" sz="1250" b="0" i="0">
             <a:solidFill>
               <a:schemeClr val="dk1"/>
             </a:solidFill>
@@ -3502,10 +3514,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3850,7 +3858,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
@@ -3861,34 +3869,34 @@
       <c r="G1" s="3"/>
       <c r="H1" s="3"/>
       <c r="I1" s="19"/>
-      <c r="J1" s="44" t="s">
+      <c r="J1" s="28" t="s">
         <v>65</v>
       </c>
       <c r="K1" s="3"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="45" t="s">
+      <c r="B2" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="44" t="s">
+      <c r="C2" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="44" t="s">
+      <c r="D2" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="E2" s="46" t="s">
+      <c r="E2" s="30" t="s">
         <v>78</v>
       </c>
-      <c r="F2" s="44" t="s">
+      <c r="F2" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="G2" s="44" t="s">
+      <c r="G2" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="44" t="s">
+      <c r="H2" s="28" t="s">
         <v>5</v>
       </c>
       <c r="I2" s="1"/>
@@ -4733,35 +4741,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="44" t="s">
+      <c r="B1" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C1" s="44" t="s">
+      <c r="C1" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="44" t="s">
+      <c r="D1" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="E1" s="44" t="s">
+      <c r="E1" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="47"/>
-      <c r="G1" s="44" t="s">
+      <c r="F1" s="31"/>
+      <c r="G1" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="H1" s="44" t="s">
+      <c r="H1" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="I1" s="44" t="s">
+      <c r="I1" s="28" t="s">
         <v>54</v>
       </c>
-      <c r="J1" s="44" t="s">
+      <c r="J1" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="K1" s="47"/>
+      <c r="K1" s="31"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
@@ -5476,25 +5484,25 @@
       <c r="A33" s="17"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A34" s="54" t="s">
+      <c r="A34" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="B34" s="55" t="s">
+      <c r="B34" s="39" t="s">
         <v>55</v>
       </c>
-      <c r="C34" s="55" t="s">
+      <c r="C34" s="39" t="s">
         <v>56</v>
       </c>
-      <c r="D34" s="55" t="s">
+      <c r="D34" s="39" t="s">
         <v>57</v>
       </c>
-      <c r="E34" s="55" t="s">
+      <c r="E34" s="39" t="s">
         <v>62</v>
       </c>
-      <c r="F34" s="55" t="s">
+      <c r="F34" s="39" t="s">
         <v>58</v>
       </c>
-      <c r="G34" s="56" t="s">
+      <c r="G34" s="40" t="s">
         <v>59</v>
       </c>
     </row>
@@ -6432,45 +6440,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="48" t="s">
+      <c r="B1" s="32" t="s">
         <v>58</v>
       </c>
-      <c r="C1" s="48" t="s">
+      <c r="C1" s="32" t="s">
         <v>59</v>
       </c>
-      <c r="D1" s="49" t="s">
+      <c r="D1" s="33" t="s">
         <v>62</v>
       </c>
-      <c r="F1" s="44" t="s">
+      <c r="F1" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="G1" s="44" t="s">
+      <c r="G1" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="H1" s="44" t="s">
+      <c r="H1" s="28" t="s">
         <v>54</v>
       </c>
-      <c r="I1" s="44" t="s">
+      <c r="I1" s="28" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="51" t="str">
+      <c r="A2" s="35" t="str">
         <f xml:space="preserve"> Calculations!A48</f>
         <v>Los Angeles Lakers</v>
       </c>
-      <c r="B2" s="52">
+      <c r="B2" s="36">
         <f>Calculations!F48</f>
         <v>7.1999999999999993</v>
       </c>
-      <c r="C2" s="53">
+      <c r="C2" s="37">
         <f>Calculations!G48</f>
         <v>1</v>
       </c>
-      <c r="D2" s="53">
+      <c r="D2" s="37">
         <f>Calculations!E48</f>
         <v>6</v>
       </c>
@@ -6492,7 +6500,7 @@
         <f xml:space="preserve"> Calculations!A54</f>
         <v>New York Knicks</v>
       </c>
-      <c r="B3" s="50">
+      <c r="B3" s="34">
         <f>Calculations!F54</f>
         <v>7.65</v>
       </c>
@@ -6522,7 +6530,7 @@
         <f xml:space="preserve"> Calculations!A36</f>
         <v>Boston Celtics</v>
       </c>
-      <c r="B4" s="50">
+      <c r="B4" s="34">
         <f>Calculations!F36</f>
         <v>8.0499999999999989</v>
       </c>
@@ -6552,7 +6560,7 @@
         <f xml:space="preserve"> Calculations!A61</f>
         <v>San Antonio Spurs</v>
       </c>
-      <c r="B5" s="50">
+      <c r="B5" s="34">
         <f>Calculations!F61</f>
         <v>8.8999999999999986</v>
       </c>
@@ -6582,7 +6590,7 @@
         <f xml:space="preserve"> Calculations!A45</f>
         <v>Houston Rockets</v>
       </c>
-      <c r="B6" s="50">
+      <c r="B6" s="34">
         <f>Calculations!F45</f>
         <v>9.35</v>
       </c>
@@ -6612,7 +6620,7 @@
         <f xml:space="preserve"> Calculations!A35</f>
         <v>Atlanta Hawks</v>
       </c>
-      <c r="B7" s="50">
+      <c r="B7" s="34">
         <f>Calculations!F35</f>
         <v>9.8000000000000007</v>
       </c>
@@ -6642,7 +6650,7 @@
         <f xml:space="preserve"> Calculations!A55</f>
         <v>Oklahoma City Thunder</v>
       </c>
-      <c r="B8" s="50">
+      <c r="B8" s="34">
         <f>Calculations!F55</f>
         <v>10.899999999999999</v>
       </c>
@@ -6660,7 +6668,7 @@
         <f xml:space="preserve"> Calculations!A57</f>
         <v>Philadelphia 76ers</v>
       </c>
-      <c r="B9" s="50">
+      <c r="B9" s="34">
         <f>Calculations!F57</f>
         <v>11.5</v>
       </c>
@@ -6678,7 +6686,7 @@
         <f xml:space="preserve"> Calculations!A47</f>
         <v>Los Angeles Clippers</v>
       </c>
-      <c r="B10" s="50">
+      <c r="B10" s="34">
         <f>Calculations!F47</f>
         <v>12.149999999999999</v>
       </c>
@@ -6696,7 +6704,7 @@
         <f xml:space="preserve"> Calculations!A44</f>
         <v>Golden State Warriors</v>
       </c>
-      <c r="B11" s="50">
+      <c r="B11" s="34">
         <f>Calculations!F44</f>
         <v>12.35</v>
       </c>
@@ -6714,7 +6722,7 @@
         <f xml:space="preserve"> Calculations!A42</f>
         <v>Denver Nuggets</v>
       </c>
-      <c r="B12" s="50">
+      <c r="B12" s="34">
         <f>Calculations!F42</f>
         <v>13.25</v>
       </c>
@@ -6732,7 +6740,7 @@
         <f xml:space="preserve"> Calculations!A58</f>
         <v>Phoenix Suns</v>
       </c>
-      <c r="B13" s="50">
+      <c r="B13" s="34">
         <f>Calculations!F58</f>
         <v>13.75</v>
       </c>
@@ -6750,7 +6758,7 @@
         <f xml:space="preserve"> Calculations!A43</f>
         <v>Detroit Pistons</v>
       </c>
-      <c r="B14" s="50">
+      <c r="B14" s="34">
         <f>Calculations!F43</f>
         <v>13.95</v>
       </c>
@@ -6768,7 +6776,7 @@
         <f xml:space="preserve"> Calculations!A62</f>
         <v>Toronto Raptors</v>
       </c>
-      <c r="B15" s="50">
+      <c r="B15" s="34">
         <f>Calculations!F62</f>
         <v>14.45</v>
       </c>
@@ -6786,7 +6794,7 @@
         <f xml:space="preserve"> Calculations!A40</f>
         <v>Cleveland Cavaliers</v>
       </c>
-      <c r="B16" s="50">
+      <c r="B16" s="34">
         <f>Calculations!F40</f>
         <v>14.45</v>
       </c>
@@ -6804,7 +6812,7 @@
         <f xml:space="preserve"> Calculations!A50</f>
         <v>Miami Heat</v>
       </c>
-      <c r="B17" s="50">
+      <c r="B17" s="34">
         <f>Calculations!F50</f>
         <v>15.35</v>
       </c>
@@ -6822,7 +6830,7 @@
         <f xml:space="preserve"> Calculations!A37</f>
         <v>Brooklyn Nets</v>
       </c>
-      <c r="B18" s="50">
+      <c r="B18" s="34">
         <f>Calculations!F37</f>
         <v>15.549999999999999</v>
       </c>
@@ -6840,7 +6848,7 @@
         <f xml:space="preserve"> Calculations!A39</f>
         <v>Chicago Bulls</v>
       </c>
-      <c r="B19" s="50">
+      <c r="B19" s="34">
         <f>Calculations!F39</f>
         <v>16</v>
       </c>
@@ -6858,7 +6866,7 @@
         <f xml:space="preserve"> Calculations!A38</f>
         <v>Charlotte Hornets</v>
       </c>
-      <c r="B20" s="50">
+      <c r="B20" s="34">
         <f>Calculations!F38</f>
         <v>17.2</v>
       </c>
@@ -6876,7 +6884,7 @@
         <f xml:space="preserve"> Calculations!A51</f>
         <v>Milwaukee Bucks</v>
       </c>
-      <c r="B21" s="50">
+      <c r="B21" s="34">
         <f>Calculations!F51</f>
         <v>17.850000000000001</v>
       </c>
@@ -6894,7 +6902,7 @@
         <f xml:space="preserve"> Calculations!A41</f>
         <v>Dallas Mavericks</v>
       </c>
-      <c r="B22" s="50">
+      <c r="B22" s="34">
         <f>Calculations!F41</f>
         <v>18.350000000000001</v>
       </c>
@@ -6912,7 +6920,7 @@
         <f xml:space="preserve"> Calculations!A56</f>
         <v>Orlando Magic</v>
       </c>
-      <c r="B23" s="50">
+      <c r="B23" s="34">
         <f>Calculations!F56</f>
         <v>19</v>
       </c>
@@ -6930,7 +6938,7 @@
         <f xml:space="preserve"> Calculations!A59</f>
         <v>Portland Trail Blazers</v>
       </c>
-      <c r="B24" s="50">
+      <c r="B24" s="34">
         <f>Calculations!F59</f>
         <v>19.2</v>
       </c>
@@ -6948,7 +6956,7 @@
         <f xml:space="preserve"> Calculations!A63</f>
         <v>Utah Jazz</v>
       </c>
-      <c r="B25" s="50">
+      <c r="B25" s="34">
         <f>Calculations!F63</f>
         <v>19.850000000000001</v>
       </c>
@@ -6966,7 +6974,7 @@
         <f xml:space="preserve"> Calculations!A49</f>
         <v>Memphis Grizzlies</v>
       </c>
-      <c r="B26" s="50">
+      <c r="B26" s="34">
         <f>Calculations!F49</f>
         <v>20.05</v>
       </c>
@@ -6984,7 +6992,7 @@
         <f xml:space="preserve"> Calculations!A52</f>
         <v>Minnesota Timberwolves</v>
       </c>
-      <c r="B27" s="50">
+      <c r="B27" s="34">
         <f>Calculations!F52</f>
         <v>20.65</v>
       </c>
@@ -7002,7 +7010,7 @@
         <f xml:space="preserve"> Calculations!A46</f>
         <v>Indiana Pacers</v>
       </c>
-      <c r="B28" s="50">
+      <c r="B28" s="34">
         <f>Calculations!F46</f>
         <v>23.75</v>
       </c>
@@ -7020,7 +7028,7 @@
         <f xml:space="preserve"> Calculations!A60</f>
         <v>Sacramento Kings</v>
       </c>
-      <c r="B29" s="50">
+      <c r="B29" s="34">
         <f>Calculations!F60</f>
         <v>23.75</v>
       </c>
@@ -7038,7 +7046,7 @@
         <f xml:space="preserve"> Calculations!A53</f>
         <v>New Orleans Pelicans</v>
       </c>
-      <c r="B30" s="50">
+      <c r="B30" s="34">
         <f>Calculations!F53</f>
         <v>24.199999999999996</v>
       </c>
@@ -7056,7 +7064,7 @@
         <f xml:space="preserve"> Calculations!A64</f>
         <v>Washington Wizards</v>
       </c>
-      <c r="B31" s="50">
+      <c r="B31" s="34">
         <f>Calculations!F64</f>
         <v>24.3</v>
       </c>
@@ -7095,152 +7103,156 @@
     <col min="11" max="11" width="19.5" style="3" customWidth="1"/>
     <col min="12" max="12" width="10.83203125" style="3"/>
     <col min="13" max="13" width="12.5" style="3" customWidth="1"/>
-    <col min="14" max="14" width="33.33203125" style="3" customWidth="1"/>
+    <col min="14" max="14" width="33.5" style="3" customWidth="1"/>
     <col min="15" max="16384" width="10.83203125" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="61" t="s">
-        <v>79</v>
-      </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
+      <c r="A1" s="42"/>
+      <c r="B1" s="42" t="s">
+        <v>95</v>
+      </c>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="42"/>
+      <c r="I1" s="42"/>
+      <c r="J1" s="42"/>
     </row>
     <row r="2" spans="1:18" ht="21" x14ac:dyDescent="0.25">
-      <c r="A2" s="57"/>
-      <c r="B2" s="60" t="s">
-        <v>95</v>
-      </c>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
+      <c r="A2" s="41"/>
+      <c r="B2" s="46" t="s">
+        <v>94</v>
+      </c>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="B4" s="40" t="s">
+      <c r="B4" s="43" t="s">
         <v>73</v>
       </c>
-      <c r="C4" s="41"/>
-      <c r="D4" s="42"/>
-      <c r="F4" s="40" t="s">
+      <c r="C4" s="44"/>
+      <c r="D4" s="45"/>
+      <c r="F4" s="43" t="s">
         <v>74</v>
       </c>
-      <c r="G4" s="41"/>
-      <c r="H4" s="42"/>
-      <c r="J4" s="40" t="s">
+      <c r="G4" s="44"/>
+      <c r="H4" s="45"/>
+      <c r="J4" s="43" t="s">
         <v>75</v>
       </c>
-      <c r="K4" s="41"/>
-      <c r="L4" s="42"/>
-      <c r="N4" s="59" t="s">
+      <c r="K4" s="44"/>
+      <c r="L4" s="45"/>
+      <c r="N4" s="27" t="s">
         <v>76</v>
       </c>
-      <c r="P4" s="43" t="s">
+      <c r="P4" s="48" t="s">
         <v>77</v>
       </c>
-      <c r="Q4" s="43"/>
-      <c r="R4" s="43"/>
+      <c r="Q4" s="48"/>
+      <c r="R4" s="48"/>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="B5" s="28" t="str">
+      <c r="B5" s="50" t="str">
         <f>Rankings!A2</f>
         <v>Los Angeles Lakers</v>
       </c>
-      <c r="C5" s="29"/>
-      <c r="D5" s="30"/>
-      <c r="F5" s="28" t="str">
+      <c r="C5" s="51"/>
+      <c r="D5" s="52"/>
+      <c r="F5" s="50" t="str">
         <f>INDEX(Calculations!$A$35:$A$64,MATCH(1,Calculations!$C$35:$C$64,0))</f>
         <v>Oklahoma City Thunder</v>
       </c>
-      <c r="G5" s="29"/>
-      <c r="H5" s="30"/>
-      <c r="J5" s="28" t="str">
+      <c r="G5" s="51"/>
+      <c r="H5" s="52"/>
+      <c r="J5" s="50" t="str">
         <f>INDEX(Calculations!$A$35:$A$64,MATCH(1,Calculations!$D$35:$D$64,0))</f>
         <v>Golden State Warriors</v>
       </c>
-      <c r="K5" s="29"/>
-      <c r="L5" s="30"/>
-      <c r="N5" s="28" t="str">
+      <c r="K5" s="51"/>
+      <c r="L5" s="52"/>
+      <c r="N5" s="50" t="str">
         <f>INDEX(Calculations!$A$2:$A$31,MATCH(MAX(Calculations!$E$2:$E$31),Calculations!$E$2:$E$31,0))</f>
         <v>Oklahoma City Thunder</v>
       </c>
-      <c r="P5" s="34">
+      <c r="P5" s="57">
         <f>AVERAGE(Data!$B$3:$B$32)/1000000</f>
         <v>197.90667206666666</v>
       </c>
-      <c r="Q5" s="35"/>
-      <c r="R5" s="36"/>
+      <c r="Q5" s="58"/>
+      <c r="R5" s="59"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="B6" s="31"/>
-      <c r="C6" s="32"/>
-      <c r="D6" s="33"/>
-      <c r="F6" s="31"/>
-      <c r="G6" s="32"/>
-      <c r="H6" s="33"/>
-      <c r="J6" s="31"/>
-      <c r="K6" s="32"/>
-      <c r="L6" s="33"/>
-      <c r="N6" s="31"/>
-      <c r="P6" s="37"/>
-      <c r="Q6" s="38"/>
-      <c r="R6" s="39"/>
+      <c r="B6" s="53"/>
+      <c r="C6" s="54"/>
+      <c r="D6" s="55"/>
+      <c r="F6" s="53"/>
+      <c r="G6" s="54"/>
+      <c r="H6" s="55"/>
+      <c r="J6" s="53"/>
+      <c r="K6" s="54"/>
+      <c r="L6" s="55"/>
+      <c r="N6" s="53"/>
+      <c r="P6" s="60"/>
+      <c r="Q6" s="61"/>
+      <c r="R6" s="62"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="N7" s="62">
+      <c r="N7" s="56">
         <f>MAX(Calculations!$E$2:$E$31)</f>
         <v>0.78</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="B8" s="25" t="s">
+      <c r="B8" s="49" t="s">
+        <v>80</v>
+      </c>
+      <c r="C8" s="49"/>
+      <c r="D8" s="49"/>
+      <c r="E8" s="49"/>
+      <c r="J8" s="49" t="s">
         <v>81</v>
       </c>
-      <c r="C8" s="25"/>
-      <c r="D8" s="25"/>
-      <c r="E8" s="25"/>
-      <c r="J8" s="25" t="s">
+      <c r="K8" s="49"/>
+      <c r="L8" s="49"/>
+      <c r="M8" s="49"/>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B9" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="C9" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="D9" s="28" t="s">
+        <v>58</v>
+      </c>
+      <c r="E9" s="28" t="s">
+        <v>62</v>
+      </c>
+      <c r="F9" s="28" t="s">
         <v>82</v>
       </c>
-      <c r="K8" s="25"/>
-      <c r="L8" s="25"/>
-      <c r="M8" s="25"/>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="B9" s="44" t="s">
-        <v>80</v>
-      </c>
-      <c r="C9" s="44" t="s">
+      <c r="J9" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="K9" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="D9" s="44" t="s">
+      <c r="L9" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="E9" s="44" t="s">
+      <c r="M9" s="28" t="s">
         <v>62</v>
       </c>
-      <c r="F9" s="44" t="s">
+      <c r="N9" s="28" t="s">
         <v>83</v>
-      </c>
-      <c r="J9" s="44" t="s">
-        <v>80</v>
-      </c>
-      <c r="K9" s="44" t="s">
-        <v>1</v>
-      </c>
-      <c r="L9" s="44" t="s">
-        <v>58</v>
-      </c>
-      <c r="M9" s="44" t="s">
-        <v>62</v>
-      </c>
-      <c r="N9" s="44" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="10" spans="1:18" ht="16" x14ac:dyDescent="0.2">
@@ -7259,8 +7271,8 @@
         <f>Rankings!D2</f>
         <v>6</v>
       </c>
-      <c r="F10" s="26" t="s">
-        <v>85</v>
+      <c r="F10" s="25" t="s">
+        <v>84</v>
       </c>
       <c r="J10" s="3">
         <v>26</v>
@@ -7277,8 +7289,8 @@
         <f>Rankings!D27</f>
         <v>10</v>
       </c>
-      <c r="N10" s="27" t="s">
-        <v>90</v>
+      <c r="N10" s="26" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.2">
@@ -7297,8 +7309,8 @@
         <f>Rankings!D3</f>
         <v>6</v>
       </c>
-      <c r="F11" s="27" t="s">
-        <v>86</v>
+      <c r="F11" s="26" t="s">
+        <v>85</v>
       </c>
       <c r="J11" s="3">
         <v>27</v>
@@ -7315,8 +7327,8 @@
         <f>Rankings!D28</f>
         <v>29</v>
       </c>
-      <c r="N11" s="27" t="s">
-        <v>91</v>
+      <c r="N11" s="26" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.2">
@@ -7335,8 +7347,8 @@
         <f>Rankings!D4</f>
         <v>4</v>
       </c>
-      <c r="F12" s="27" t="s">
-        <v>87</v>
+      <c r="F12" s="26" t="s">
+        <v>86</v>
       </c>
       <c r="J12" s="3">
         <v>27</v>
@@ -7353,8 +7365,8 @@
         <f>Rankings!D29</f>
         <v>26</v>
       </c>
-      <c r="N12" s="27" t="s">
-        <v>92</v>
+      <c r="N12" s="26" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.2">
@@ -7373,8 +7385,8 @@
         <f>Rankings!D5</f>
         <v>2</v>
       </c>
-      <c r="F13" s="27" t="s">
-        <v>88</v>
+      <c r="F13" s="26" t="s">
+        <v>87</v>
       </c>
       <c r="J13" s="3">
         <v>29</v>
@@ -7391,8 +7403,8 @@
         <f>Rankings!D30</f>
         <v>23</v>
       </c>
-      <c r="N13" s="27" t="s">
-        <v>93</v>
+      <c r="N13" s="26" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.2">
@@ -7411,8 +7423,8 @@
         <f>Rankings!D6</f>
         <v>8</v>
       </c>
-      <c r="F14" s="27" t="s">
-        <v>89</v>
+      <c r="F14" s="26" t="s">
+        <v>88</v>
       </c>
       <c r="J14" s="3">
         <v>30</v>
@@ -7429,13 +7441,12 @@
         <f>Rankings!D31</f>
         <v>30</v>
       </c>
-      <c r="N14" s="27" t="s">
-        <v>94</v>
+      <c r="N14" s="26" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
-    <mergeCell ref="A1:F1"/>
+  <mergeCells count="12">
     <mergeCell ref="B2:H2"/>
     <mergeCell ref="N5:N6"/>
     <mergeCell ref="P4:R4"/>

</xml_diff>